<commit_message>
Aclara contrafactual agregado en resumen
</commit_message>
<xml_diff>
--- a/outputs/ptf_pesos_vbp_20260727_financieras/anex-PTF-Productividad-2025_con_calculos_CJC.xlsx
+++ b/outputs/ptf_pesos_vbp_20260727_financieras/anex-PTF-Productividad-2025_con_calculos_CJC.xlsx
@@ -2,36 +2,36 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Índice" sheetId="9" r:id="Rf3450af4fe364ea8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 1" sheetId="25" r:id="Ra8efae165e644adb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 2" sheetId="6" r:id="R19500bc763454be3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 3" sheetId="8" r:id="R578ef0327217401c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 4" sheetId="31" r:id="R6880ffd1e09c40a8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 5" sheetId="32" r:id="R55af59dd4e93421b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 6" sheetId="33" r:id="R1892449c93534a0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 7" sheetId="34" r:id="Re24cd333fe354f96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 8" sheetId="35" r:id="R0df7fa157e5348cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 9" sheetId="36" r:id="R6b636a1262ad4834"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 10" sheetId="37" r:id="R31072b711a46426e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 11" sheetId="38" r:id="R26edea4076974219"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 12" sheetId="39" r:id="R1649065fdbad474d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 13" sheetId="40" r:id="Rf344d39e74e84abd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 14" sheetId="41" r:id="R6e1eb21921534969"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 15" sheetId="42" r:id="R64986a2a00db45fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 16" sheetId="43" r:id="Re1860aec50084d2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 17" sheetId="44" r:id="R5b36f9d89b9b4e15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 18" sheetId="45" r:id="Rb1155f9f9f0c477b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 19" sheetId="46" r:id="Raaa78101a7a8401f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 20" sheetId="47" r:id="Re99bf51fd5a44659"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 21" sheetId="28" r:id="Ra4623d881c0e4be5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 22" sheetId="29" r:id="Rf52c218504074d91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 23" sheetId="30" r:id="R713a45e1ec02438f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CJC Guía" sheetId="48" r:id="Rb1f758dea3a44120"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CJC VA total" sheetId="49" r:id="Rcedaa86eca09460f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CJC PTF actividad" sheetId="50" r:id="R4280466579b54dd1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CJC Pesos VBP" sheetId="51" r:id="Rb00b9edd3e5a45b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CJC Contribuciones" sheetId="52" r:id="Rbecb759bfcc843e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CJC Figuras" sheetId="53" r:id="R703def2ca1c94904"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Índice" sheetId="9" r:id="R8ec7996a47d24906"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 1" sheetId="25" r:id="Ra6093348652e4178"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 2" sheetId="6" r:id="R852dadac678a42d0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 3" sheetId="8" r:id="R357d715568864668"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 4" sheetId="31" r:id="R2f233308d6664573"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 5" sheetId="32" r:id="R3c64e8e357ce49dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 6" sheetId="33" r:id="R0afb98dfc5184b44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 7" sheetId="34" r:id="Ra71c93a6a8514620"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 8" sheetId="35" r:id="Ra2dff26601d64467"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 9" sheetId="36" r:id="R4049836f4abb4e54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 10" sheetId="37" r:id="R4551a960dc1d4390"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 11" sheetId="38" r:id="R6b6612c40fd64a4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 12" sheetId="39" r:id="R1d5d2cfa5e884e3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 13" sheetId="40" r:id="Ra948cdaa74754a88"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 14" sheetId="41" r:id="Rbc92309f908d431a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 15" sheetId="42" r:id="R8e11e02b6e7e4274"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 16" sheetId="43" r:id="Rd5ba6cac2a894ec5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 17" sheetId="44" r:id="R375b25f26cd54d74"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 18" sheetId="45" r:id="R6530f71029464cd0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 19" sheetId="46" r:id="R94552d550a4b487f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 20" sheetId="47" r:id="Rc1643da70ea04704"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 21" sheetId="28" r:id="R3533d02d55c842a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 22" sheetId="29" r:id="R26457df361174a3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadro 23" sheetId="30" r:id="Rfb6ab6ad3d844f33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CJC Guía" sheetId="48" r:id="R32f393188e474f19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CJC VA total" sheetId="49" r:id="R0269529c21cc484b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CJC PTF actividad" sheetId="50" r:id="R4501b1fd02b44f60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CJC Pesos VBP" sheetId="51" r:id="R9da1f234f2714f8d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CJC Contribuciones" sheetId="52" r:id="R5e68c38bd89d40a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CJC Figuras" sheetId="53" r:id="Re68a58da156e493e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2621,7 +2621,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R96c7cda281ef48e8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R80b1ae000cc44758"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2653,7 +2653,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R925e59295dba4fe1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbdb4df35469e4c45"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2685,7 +2685,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra02819f6bdc94e1a"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0aa6fd35213c4ff2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2717,7 +2717,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R52dc8c88f9cc426a"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd3a22ea8cc2e4e33"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2749,7 +2749,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7122253eda0b4fee"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7b5b8fda538e4c0d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2781,7 +2781,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2983246681f74572"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra2719d1d509840da"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2813,7 +2813,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R4b7e0c83e6bd4862"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra057b484128e4531"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2845,7 +2845,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R25505d4a29524886"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf953e596e4e140a1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2877,7 +2877,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R458397e60f054882"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf319dffd756d4079"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2909,7 +2909,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R80415497cfb44e19"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rb0c4a2834a8f4179"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2941,7 +2941,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5d26a83a3f5d40bf"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R71e175e34a0a4be5"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -2973,7 +2973,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2ea8d9a058514db7"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0d64bfaf9bd84f9d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3005,7 +3005,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rccde0e3e320d46cd"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9b03c50337624c95"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3037,7 +3037,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R879e71d1b4bb48c4"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R13b6f258c4dc4dd9"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3069,7 +3069,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf43d8eba09cf453f"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7c558156565e42ef"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3101,7 +3101,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rcf332fe39224407d"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re2ccfa78f9d54f82"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3133,7 +3133,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9ee693b35fa6475a"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rde26df89eb674cd0"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3165,7 +3165,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R177210f06b2048c9"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R7acda2a1f1994370"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3197,7 +3197,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R069a01b5c63e4368"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rabdd60a11ac34244"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3229,7 +3229,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1ddee9cbf26e4998"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf8d3019d71964df6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3261,7 +3261,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9c16a91180ed4f6e"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R057a9368f6e24238"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3293,7 +3293,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf7a991008de549c2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1790235235144a3c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3330,7 +3330,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R45e0dae248214b1f"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9b0185fb179449e4"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3362,7 +3362,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R145145c4a36d47b5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2ea927d7daf0472d"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3394,7 +3394,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R68b03560e5974ba6"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd0ebb51e73b14c29"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3426,7 +3426,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R93beac980e6d4fc7"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rf2ee5a22168549e1"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3458,7 +3458,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R54cdf42ef43d41fe"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R763f41a476084737"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3490,7 +3490,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9f5b5852a2b44943"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R55fa9f7689f84e5f"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3527,7 +3527,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R96ef9b71de4b48a1"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra936f3d7ee324ab2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3554,7 +3554,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R41466aa520e34517"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd8b29c2218dd4496"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3591,7 +3591,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R49a0d6426dfc47fb"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8551159a70634280"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3618,7 +3618,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra5fc292b4a9d4bf9"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R528cf7930e7843a6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3655,7 +3655,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R016d3b9486ce4315"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd749844163314d77"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3682,7 +3682,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R64708e6d3f0b475f"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R8324a168ed8740c9"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3714,7 +3714,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R137dee00f19c4966"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R95b87bf8ef524551"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3746,7 +3746,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re3c623096f124867"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R9621f11d7f394440"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3778,7 +3778,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbbbcb05c2fd742a5"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R919683d415f64ace"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3810,7 +3810,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Ra482f6ebcaf741f2"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R1b585e2c3275409a"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3842,7 +3842,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R2448e9604f154dff"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rfd86a23f96c244ae"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3874,7 +3874,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd7551b784dd742c8"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R5d5cb752904d4887"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3906,7 +3906,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd8470cfd6ef2452f"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R539de7ae6ca449f8"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3938,7 +3938,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd4df6a41a58241b4"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R78f7d3e87e5a4ba2"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -3970,7 +3970,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R180cf6edcae24240"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R628ce65be2474f6f"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -4002,7 +4002,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rd5189b46498347ee"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R53818dccffa84dea"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -4034,7 +4034,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rfc0c8cb9ff404178"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0bc2649ed2a44df6"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -4066,7 +4066,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rc696ab3ea28b4a20"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R04a18d2c444b4d69"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -4098,7 +4098,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Rbaedbc4e04914cc7"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="Re474c6c189724b4c"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -4130,7 +4130,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R0e949851b8f9463a"/>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" r:embed="R27ffc1325c544b08"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -5104,7 +5104,7 @@
     <x:hyperlink ref="B32" location="'Cuadro 23'!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R06eeb14c0c1c4a23"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ec0942fdef54721"/>
 </x:worksheet>
 </file>
 
@@ -6060,7 +6060,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d5aed017ea7400f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38304a1b40d445aa"/>
 </x:worksheet>
 </file>
 
@@ -7016,7 +7016,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a0e397ac7904b7f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0ab8f19e131942b6"/>
 </x:worksheet>
 </file>
 
@@ -7972,7 +7972,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R531134ad0bc64e43"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf2d5117f4c774c15"/>
 </x:worksheet>
 </file>
 
@@ -8928,7 +8928,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c3175a2aa1a4af1"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff2d31abe8034b28"/>
 </x:worksheet>
 </file>
 
@@ -9884,7 +9884,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfbbd14c4713f4206"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6b94c43138104166"/>
 </x:worksheet>
 </file>
 
@@ -10840,7 +10840,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1f4f1d59f764a96"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R492bcf20ec6b498b"/>
 </x:worksheet>
 </file>
 
@@ -11796,7 +11796,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R61d1d43e79614e70"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rac6b3e86f2b54205"/>
 </x:worksheet>
 </file>
 
@@ -12752,7 +12752,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refd67d202167427b"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb09810e69d444bfc"/>
 </x:worksheet>
 </file>
 
@@ -13708,7 +13708,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1ee4ff6befd49d8"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8098e5d967934fb9"/>
 </x:worksheet>
 </file>
 
@@ -14664,7 +14664,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3815947881674c91"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc0b674724c674796"/>
 </x:worksheet>
 </file>
 
@@ -15407,7 +15407,7 @@
     <x:hyperlink ref="H5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R319a257236844d69"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R88ea9ce258ba4db6"/>
 </x:worksheet>
 </file>
 
@@ -16363,7 +16363,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4326ee5d74349b9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R76f693cd0ee44e87"/>
 </x:worksheet>
 </file>
 
@@ -17319,7 +17319,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e95ecf95ef045a3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf119ee129dd1468d"/>
 </x:worksheet>
 </file>
 
@@ -18276,7 +18276,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a7aaf07e52c4151"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R788e0e994f494962"/>
 </x:worksheet>
 </file>
 
@@ -19239,7 +19239,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85a7407fcf704295"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ac7ce851ea940c7"/>
 </x:worksheet>
 </file>
 
@@ -20224,7 +20224,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra28e623e00574c95"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R867830bd841f4113"/>
 </x:worksheet>
 </file>
 
@@ -31242,7 +31242,7 @@
     <x:hyperlink ref="L5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ce90747a13b4cca"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R13a71838710f4c6b"/>
 </x:worksheet>
 </file>
 
@@ -32386,7 +32386,7 @@
     <x:hyperlink ref="K5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re347cfd7d2464d9d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e017e473d814a45"/>
 </x:worksheet>
 </file>
 
@@ -33342,7 +33342,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb4e1be08de94b8f"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rde439f33bdb34bc7"/>
 </x:worksheet>
 </file>
 
@@ -34298,7 +34298,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3b138c7fb0594dff"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfbe922304ff4ceb"/>
 </x:worksheet>
 </file>
 
@@ -35254,7 +35254,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R903c536aedba4c14"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2e46cede05242be"/>
 </x:worksheet>
 </file>
 
@@ -36210,7 +36210,7 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07f679056e734c45"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb510e444f8114144"/>
 </x:worksheet>
 </file>
 
@@ -37166,6 +37166,6 @@
     <x:hyperlink ref="P5" location="Índice!A1"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cbfdd939af44e72"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0852efdba4344dc3"/>
 </x:worksheet>
 </file>
</xml_diff>